<commit_message>
Registration workbook template: no signature rows, logo centred at the top of every sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/registration-template.xlsx
+++ b/registration-template.xlsx
@@ -24,29 +24,29 @@
     <sheet name="التاسع ذكور" sheetId="14" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">الأول!$A$1:$K$44</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">الأول!$A$1:$K$39</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">الأول!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="10" name="_xlnm.Print_Area" vbProcedure="false">'التاسع بنات'!$A$1:$K$38</definedName>
+    <definedName function="false" hidden="false" localSheetId="10" name="_xlnm.Print_Area" vbProcedure="false">'التاسع بنات'!$A$1:$K$33</definedName>
     <definedName function="false" hidden="false" localSheetId="10" name="_xlnm.Print_Titles" vbProcedure="false">'التاسع بنات'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="13" name="_xlnm.Print_Area" vbProcedure="false">'التاسع ذكور'!$A$1:$K$42</definedName>
+    <definedName function="false" hidden="false" localSheetId="13" name="_xlnm.Print_Area" vbProcedure="false">'التاسع ذكور'!$A$1:$K$37</definedName>
     <definedName function="false" hidden="false" localSheetId="13" name="_xlnm.Print_Titles" vbProcedure="false">'التاسع ذكور'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">الثالث!$A$1:$K$44</definedName>
+    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">الثالث!$A$1:$K$39</definedName>
     <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Titles" vbProcedure="false">الثالث!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Area" vbProcedure="false">'الثامن بنات'!$A$1:$K$34</definedName>
+    <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Area" vbProcedure="false">'الثامن بنات'!$A$1:$K$29</definedName>
     <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Titles" vbProcedure="false">'الثامن بنات'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="12" name="_xlnm.Print_Area" vbProcedure="false">'الثامن ذكور'!$A$1:$K$34</definedName>
+    <definedName function="false" hidden="false" localSheetId="12" name="_xlnm.Print_Area" vbProcedure="false">'الثامن ذكور'!$A$1:$K$29</definedName>
     <definedName function="false" hidden="false" localSheetId="12" name="_xlnm.Print_Titles" vbProcedure="false">'الثامن ذكور'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">الثاني!$A$1:$K$34</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">الثاني!$A$1:$K$29</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">الثاني!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Area" vbProcedure="false">الخامس!$A$1:$K$34</definedName>
+    <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Area" vbProcedure="false">الخامس!$A$1:$K$29</definedName>
     <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Titles" vbProcedure="false">الخامس!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Area" vbProcedure="false">الرابع!$A$1:$K$44</definedName>
+    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Area" vbProcedure="false">الرابع!$A$1:$K$39</definedName>
     <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Titles" vbProcedure="false">الرابع!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Area" vbProcedure="false">'السابع بنات'!$A$1:$K$38</definedName>
+    <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Area" vbProcedure="false">'السابع بنات'!$A$1:$K$33</definedName>
     <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Titles" vbProcedure="false">'السابع بنات'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="11" name="_xlnm.Print_Area" vbProcedure="false">'السابع ذكور'!$A$1:$K$34</definedName>
+    <definedName function="false" hidden="false" localSheetId="11" name="_xlnm.Print_Area" vbProcedure="false">'السابع ذكور'!$A$1:$K$29</definedName>
     <definedName function="false" hidden="false" localSheetId="11" name="_xlnm.Print_Titles" vbProcedure="false">'السابع ذكور'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Area" vbProcedure="false">السادس!$A$1:$K$34</definedName>
+    <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Area" vbProcedure="false">السادس!$A$1:$K$29</definedName>
     <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Titles" vbProcedure="false">السادس!$9:$9</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -797,19 +797,14 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>-2857320</xdr:colOff>
+      <xdr:colOff>2038350</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>247320</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="2000250" cy="1524000"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
@@ -821,8 +816,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-3139200" y="0"/>
-          <a:ext cx="2857320" cy="2171520"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="2000250" cy="1524000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -833,25 +828,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="Image 1" descr="Picture"/>
@@ -863,8 +853,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -875,25 +865,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
@@ -905,8 +890,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -917,25 +902,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="11" name="Image 1" descr="Picture"/>
@@ -947,8 +927,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -959,25 +939,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="12" name="Image 1" descr="Picture"/>
@@ -989,8 +964,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1001,25 +976,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="13" name="Image 1" descr="Picture"/>
@@ -1031,8 +1001,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1043,25 +1013,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>809625</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1073,8 +1038,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1085,25 +1050,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
@@ -1115,8 +1075,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1127,25 +1087,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Image 1" descr="Picture"/>
@@ -1157,8 +1112,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1169,25 +1124,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="4" name="Image 1" descr="Picture"/>
@@ -1199,8 +1149,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1211,25 +1161,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
@@ -1241,8 +1186,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1253,25 +1198,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="6" name="Image 1" descr="Picture"/>
@@ -1283,8 +1223,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1295,25 +1235,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Image 1" descr="Picture"/>
@@ -1325,8 +1260,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1337,25 +1272,20 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>-647280</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="952500" cy="723900"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="8" name="Image 1" descr="Picture"/>
@@ -1367,8 +1297,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="-999720" y="0"/>
-          <a:ext cx="999720" cy="761760"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="952500" cy="723900"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1379,7 +1309,7 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1650,7 +1580,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1665,10 +1595,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -2140,36 +2068,8 @@
       <c r="J29" s="34"/>
       <c r="K29" s="34"/>
     </row>
-    <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B32" s="38"/>
-      <c r="C32" s="38"/>
-      <c r="E32" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="I32" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J32" s="38"/>
-      <c r="K32" s="38"/>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="39"/>
-      <c r="B34" s="39"/>
-      <c r="C34" s="39"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="39"/>
-      <c r="I34" s="39"/>
-      <c r="J34" s="39"/>
-      <c r="K34" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -2181,12 +2081,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="E34:G34"/>
-    <mergeCell ref="I34:K34"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -2216,7 +2110,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2231,10 +2125,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -2774,36 +2666,8 @@
       <c r="J33" s="34"/>
       <c r="K33" s="34"/>
     </row>
-    <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B36" s="38"/>
-      <c r="C36" s="38"/>
-      <c r="E36" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F36" s="38"/>
-      <c r="G36" s="38"/>
-      <c r="I36" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J36" s="38"/>
-      <c r="K36" s="38"/>
-    </row>
-    <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="39"/>
-      <c r="B38" s="39"/>
-      <c r="C38" s="39"/>
-      <c r="E38" s="39"/>
-      <c r="F38" s="39"/>
-      <c r="G38" s="39"/>
-      <c r="I38" s="39"/>
-      <c r="J38" s="39"/>
-      <c r="K38" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -2815,12 +2679,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="E36:G36"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="I38:K38"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -2850,7 +2708,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2865,10 +2723,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -3340,36 +3196,8 @@
       <c r="J29" s="34"/>
       <c r="K29" s="34"/>
     </row>
-    <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B32" s="38"/>
-      <c r="C32" s="38"/>
-      <c r="E32" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="I32" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J32" s="38"/>
-      <c r="K32" s="38"/>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="39"/>
-      <c r="B34" s="39"/>
-      <c r="C34" s="39"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="39"/>
-      <c r="I34" s="39"/>
-      <c r="J34" s="39"/>
-      <c r="K34" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -3381,12 +3209,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="E34:G34"/>
-    <mergeCell ref="I34:K34"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -3416,7 +3238,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3431,10 +3253,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -3906,36 +3726,8 @@
       <c r="J29" s="34"/>
       <c r="K29" s="34"/>
     </row>
-    <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B32" s="38"/>
-      <c r="C32" s="38"/>
-      <c r="E32" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="I32" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J32" s="38"/>
-      <c r="K32" s="38"/>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="39"/>
-      <c r="B34" s="39"/>
-      <c r="C34" s="39"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="39"/>
-      <c r="I34" s="39"/>
-      <c r="J34" s="39"/>
-      <c r="K34" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -3947,12 +3739,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="E34:G34"/>
-    <mergeCell ref="I34:K34"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -3982,7 +3768,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3997,10 +3783,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -4608,36 +4392,8 @@
       <c r="J37" s="34"/>
       <c r="K37" s="34"/>
     </row>
-    <row r="40" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B40" s="38"/>
-      <c r="C40" s="38"/>
-      <c r="E40" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F40" s="38"/>
-      <c r="G40" s="38"/>
-      <c r="I40" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J40" s="38"/>
-      <c r="K40" s="38"/>
-    </row>
-    <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="39"/>
-      <c r="B42" s="39"/>
-      <c r="C42" s="39"/>
-      <c r="E42" s="39"/>
-      <c r="F42" s="39"/>
-      <c r="G42" s="39"/>
-      <c r="I42" s="39"/>
-      <c r="J42" s="39"/>
-      <c r="K42" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -4649,12 +4405,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="E40:G40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="E42:G42"/>
-    <mergeCell ref="I42:K42"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -4694,10 +4444,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="5" style="0" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -5186,7 +4934,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -5201,10 +4949,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -5800,36 +5546,8 @@
       <c r="J39" s="34"/>
       <c r="K39" s="34"/>
     </row>
-    <row r="42" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B42" s="38"/>
-      <c r="C42" s="38"/>
-      <c r="E42" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F42" s="38"/>
-      <c r="G42" s="38"/>
-      <c r="I42" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J42" s="38"/>
-      <c r="K42" s="38"/>
-    </row>
-    <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="39"/>
-      <c r="B44" s="39"/>
-      <c r="C44" s="39"/>
-      <c r="E44" s="39"/>
-      <c r="F44" s="39"/>
-      <c r="G44" s="39"/>
-      <c r="I44" s="39"/>
-      <c r="J44" s="39"/>
-      <c r="K44" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -5841,12 +5559,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="E42:G42"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="I44:K44"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -5880,7 +5592,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -5895,10 +5607,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -6344,36 +6054,8 @@
       <c r="J29" s="34"/>
       <c r="K29" s="34"/>
     </row>
-    <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B32" s="38"/>
-      <c r="C32" s="38"/>
-      <c r="E32" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="I32" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J32" s="38"/>
-      <c r="K32" s="38"/>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="39"/>
-      <c r="B34" s="39"/>
-      <c r="C34" s="39"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="39"/>
-      <c r="I34" s="39"/>
-      <c r="J34" s="39"/>
-      <c r="K34" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -6385,12 +6067,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="E34:G34"/>
-    <mergeCell ref="I34:K34"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -6424,7 +6100,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -6439,10 +6115,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -7038,36 +6712,8 @@
       <c r="J39" s="34"/>
       <c r="K39" s="34"/>
     </row>
-    <row r="42" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B42" s="38"/>
-      <c r="C42" s="38"/>
-      <c r="E42" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F42" s="38"/>
-      <c r="G42" s="38"/>
-      <c r="I42" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J42" s="38"/>
-      <c r="K42" s="38"/>
-    </row>
-    <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="39"/>
-      <c r="B44" s="39"/>
-      <c r="C44" s="39"/>
-      <c r="E44" s="39"/>
-      <c r="F44" s="39"/>
-      <c r="G44" s="39"/>
-      <c r="I44" s="39"/>
-      <c r="J44" s="39"/>
-      <c r="K44" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -7079,12 +6725,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="E42:G42"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="I44:K44"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -7118,7 +6758,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -7133,10 +6773,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -7732,36 +7370,8 @@
       <c r="J39" s="34"/>
       <c r="K39" s="34"/>
     </row>
-    <row r="42" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B42" s="38"/>
-      <c r="C42" s="38"/>
-      <c r="E42" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F42" s="38"/>
-      <c r="G42" s="38"/>
-      <c r="I42" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J42" s="38"/>
-      <c r="K42" s="38"/>
-    </row>
-    <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="39"/>
-      <c r="B44" s="39"/>
-      <c r="C44" s="39"/>
-      <c r="E44" s="39"/>
-      <c r="F44" s="39"/>
-      <c r="G44" s="39"/>
-      <c r="I44" s="39"/>
-      <c r="J44" s="39"/>
-      <c r="K44" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -7773,12 +7383,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="E42:G42"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="E44:G44"/>
-    <mergeCell ref="I44:K44"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -7812,7 +7416,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -7827,10 +7431,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -8276,36 +7878,8 @@
       <c r="J29" s="34"/>
       <c r="K29" s="34"/>
     </row>
-    <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B32" s="38"/>
-      <c r="C32" s="38"/>
-      <c r="E32" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="I32" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J32" s="38"/>
-      <c r="K32" s="38"/>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="39"/>
-      <c r="B34" s="39"/>
-      <c r="C34" s="39"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="39"/>
-      <c r="I34" s="39"/>
-      <c r="J34" s="39"/>
-      <c r="K34" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -8317,12 +7891,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="E34:G34"/>
-    <mergeCell ref="I34:K34"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -8356,7 +7924,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -8371,10 +7939,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -8820,36 +8386,8 @@
       <c r="J29" s="34"/>
       <c r="K29" s="34"/>
     </row>
-    <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B32" s="38"/>
-      <c r="C32" s="38"/>
-      <c r="E32" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F32" s="38"/>
-      <c r="G32" s="38"/>
-      <c r="I32" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J32" s="38"/>
-      <c r="K32" s="38"/>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="39"/>
-      <c r="B34" s="39"/>
-      <c r="C34" s="39"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="39"/>
-      <c r="G34" s="39"/>
-      <c r="I34" s="39"/>
-      <c r="J34" s="39"/>
-      <c r="K34" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -8861,12 +8399,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="I32:K32"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="E34:G34"/>
-    <mergeCell ref="I34:K34"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
@@ -8900,7 +8432,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -8915,10 +8447,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6" t="s">
-        <v>12</v>
-      </c>
+    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6"/>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -9458,36 +8988,8 @@
       <c r="J33" s="34"/>
       <c r="K33" s="34"/>
     </row>
-    <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B36" s="38"/>
-      <c r="C36" s="38"/>
-      <c r="E36" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F36" s="38"/>
-      <c r="G36" s="38"/>
-      <c r="I36" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="J36" s="38"/>
-      <c r="K36" s="38"/>
-    </row>
-    <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="39"/>
-      <c r="B38" s="39"/>
-      <c r="C38" s="39"/>
-      <c r="E38" s="39"/>
-      <c r="F38" s="39"/>
-      <c r="G38" s="39"/>
-      <c r="I38" s="39"/>
-      <c r="J38" s="39"/>
-      <c r="K38" s="39"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="11">
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C2:I2"/>
     <mergeCell ref="C3:I3"/>
@@ -9499,12 +9001,6 @@
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="E36:G36"/>
-    <mergeCell ref="I36:K36"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="I38:K38"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">

</xml_diff>

<commit_message>
Registration workbook: no logo, phones without +, residence column shows the city
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/registration-template.xlsx
+++ b/registration-template.xlsx
@@ -795,524 +795,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2038350</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="2000250" cy="1524000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2000250" cy="1524000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>809625</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="952500" cy="723900"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="952500" cy="723900"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -1570,7 +1052,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1595,8 +1076,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -2100,7 +1583,6 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2125,8 +1607,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -2698,7 +2182,6 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2723,8 +2206,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -3228,7 +2713,6 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3253,8 +2737,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -3758,7 +3244,6 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3783,8 +3268,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -4424,7 +3911,6 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4444,8 +3930,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="5" style="0" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -4924,7 +4412,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4949,8 +4436,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -5582,7 +5071,6 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5607,8 +5095,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -6090,7 +5580,6 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6115,8 +5604,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -6748,7 +6239,6 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6773,8 +6263,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -7406,7 +6898,6 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7431,8 +6922,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -7914,7 +7407,6 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7939,8 +7431,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -8422,7 +7916,6 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8447,8 +7940,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C1" s="6"/>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C1" s="6" t="s">
+        <v>12</v>
+      </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
@@ -9020,6 +8515,5 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;"Arial,Regular"أكاديمية الركيزة الثالثة — صفحة &amp;P من &amp;N</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Registration workbook: student's mobile column, phone numbers without '+'
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/registration-template.xlsx
+++ b/registration-template.xlsx
@@ -24,29 +24,29 @@
     <sheet name="التاسع ذكور" sheetId="14" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">الأول!$A$1:$K$39</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">الأول!$A$1:$L$39</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">الأول!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="10" name="_xlnm.Print_Area" vbProcedure="false">'التاسع بنات'!$A$1:$K$33</definedName>
+    <definedName function="false" hidden="false" localSheetId="10" name="_xlnm.Print_Area" vbProcedure="false">'التاسع بنات'!$A$1:$L$33</definedName>
     <definedName function="false" hidden="false" localSheetId="10" name="_xlnm.Print_Titles" vbProcedure="false">'التاسع بنات'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="13" name="_xlnm.Print_Area" vbProcedure="false">'التاسع ذكور'!$A$1:$K$37</definedName>
+    <definedName function="false" hidden="false" localSheetId="13" name="_xlnm.Print_Area" vbProcedure="false">'التاسع ذكور'!$A$1:$L$37</definedName>
     <definedName function="false" hidden="false" localSheetId="13" name="_xlnm.Print_Titles" vbProcedure="false">'التاسع ذكور'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">الثالث!$A$1:$K$39</definedName>
+    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">الثالث!$A$1:$L$39</definedName>
     <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Titles" vbProcedure="false">الثالث!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Area" vbProcedure="false">'الثامن بنات'!$A$1:$K$29</definedName>
+    <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Area" vbProcedure="false">'الثامن بنات'!$A$1:$L$29</definedName>
     <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Titles" vbProcedure="false">'الثامن بنات'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="12" name="_xlnm.Print_Area" vbProcedure="false">'الثامن ذكور'!$A$1:$K$29</definedName>
+    <definedName function="false" hidden="false" localSheetId="12" name="_xlnm.Print_Area" vbProcedure="false">'الثامن ذكور'!$A$1:$L$29</definedName>
     <definedName function="false" hidden="false" localSheetId="12" name="_xlnm.Print_Titles" vbProcedure="false">'الثامن ذكور'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">الثاني!$A$1:$K$29</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">الثاني!$A$1:$L$29</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">الثاني!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Area" vbProcedure="false">الخامس!$A$1:$K$29</definedName>
+    <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Area" vbProcedure="false">الخامس!$A$1:$L$29</definedName>
     <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Titles" vbProcedure="false">الخامس!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Area" vbProcedure="false">الرابع!$A$1:$K$39</definedName>
+    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Area" vbProcedure="false">الرابع!$A$1:$L$39</definedName>
     <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Titles" vbProcedure="false">الرابع!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Area" vbProcedure="false">'السابع بنات'!$A$1:$K$33</definedName>
+    <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Area" vbProcedure="false">'السابع بنات'!$A$1:$L$33</definedName>
     <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Titles" vbProcedure="false">'السابع بنات'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="11" name="_xlnm.Print_Area" vbProcedure="false">'السابع ذكور'!$A$1:$K$29</definedName>
+    <definedName function="false" hidden="false" localSheetId="11" name="_xlnm.Print_Area" vbProcedure="false">'السابع ذكور'!$A$1:$L$29</definedName>
     <definedName function="false" hidden="false" localSheetId="11" name="_xlnm.Print_Titles" vbProcedure="false">'السابع ذكور'!$9:$9</definedName>
-    <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Area" vbProcedure="false">السادس!$A$1:$K$29</definedName>
+    <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Area" vbProcedure="false">السادس!$A$1:$L$29</definedName>
     <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Titles" vbProcedure="false">السادس!$9:$9</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -1061,7 +1061,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1071,9 +1071,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1086,6 +1086,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -1097,6 +1098,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -1108,6 +1110,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -1121,6 +1124,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -1141,6 +1145,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -1204,10 +1209,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1225,8 +1235,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -1242,8 +1253,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -1259,8 +1271,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -1276,8 +1289,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -1293,8 +1307,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -1310,8 +1325,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -1327,8 +1343,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -1344,8 +1361,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -1361,8 +1379,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -1378,8 +1397,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -1395,8 +1415,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -1412,8 +1433,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -1429,8 +1451,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -1446,8 +1469,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -1463,8 +1487,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -1480,8 +1505,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -1497,8 +1523,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -1514,8 +1541,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -1531,8 +1559,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -1548,18 +1577,19 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
@@ -1592,7 +1622,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1602,9 +1632,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1617,6 +1647,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -1628,6 +1659,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -1639,6 +1671,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -1652,6 +1685,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -1672,6 +1706,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -1735,10 +1770,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1756,8 +1796,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -1773,8 +1814,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -1790,8 +1832,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -1807,8 +1850,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -1824,8 +1868,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -1841,8 +1886,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -1858,8 +1904,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -1875,8 +1922,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -1892,8 +1940,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -1909,8 +1958,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -1926,8 +1976,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -1943,8 +1994,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -1960,8 +2012,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -1977,8 +2030,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -1994,8 +2048,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -2011,8 +2066,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -2028,8 +2084,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -2045,8 +2102,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -2062,8 +2120,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -2079,8 +2138,9 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="n">
@@ -2096,8 +2156,9 @@
       <c r="G30" s="31"/>
       <c r="H30" s="33"/>
       <c r="I30" s="33"/>
-      <c r="J30" s="30"/>
+      <c r="J30" s="33"/>
       <c r="K30" s="30"/>
+      <c r="L30" s="30"/>
     </row>
     <row r="31" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="n">
@@ -2113,8 +2174,9 @@
       <c r="G31" s="35"/>
       <c r="H31" s="37"/>
       <c r="I31" s="37"/>
-      <c r="J31" s="34"/>
+      <c r="J31" s="37"/>
       <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
     </row>
     <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="n">
@@ -2130,8 +2192,9 @@
       <c r="G32" s="31"/>
       <c r="H32" s="33"/>
       <c r="I32" s="33"/>
-      <c r="J32" s="30"/>
+      <c r="J32" s="33"/>
       <c r="K32" s="30"/>
+      <c r="L32" s="30"/>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="n">
@@ -2147,18 +2210,19 @@
       <c r="G33" s="35"/>
       <c r="H33" s="37"/>
       <c r="I33" s="37"/>
-      <c r="J33" s="34"/>
+      <c r="J33" s="37"/>
       <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
@@ -2191,7 +2255,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2201,9 +2265,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2216,6 +2280,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -2227,6 +2292,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -2238,6 +2304,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -2251,6 +2318,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -2271,6 +2339,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -2334,10 +2403,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2355,8 +2429,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -2372,8 +2447,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -2389,8 +2465,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -2406,8 +2483,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -2423,8 +2501,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -2440,8 +2519,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -2457,8 +2537,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -2474,8 +2555,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -2491,8 +2573,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -2508,8 +2591,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -2525,8 +2609,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -2542,8 +2627,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -2559,8 +2645,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -2576,8 +2663,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -2593,8 +2681,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -2610,8 +2699,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -2627,8 +2717,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -2644,8 +2735,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -2661,8 +2753,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -2678,18 +2771,19 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
@@ -2722,7 +2816,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2732,9 +2826,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2747,6 +2841,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -2758,6 +2853,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -2769,6 +2865,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -2782,6 +2879,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -2802,6 +2900,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -2865,10 +2964,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2886,8 +2990,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -2903,8 +3008,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -2920,8 +3026,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -2937,8 +3044,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -2954,8 +3062,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -2971,8 +3080,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -2988,8 +3098,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -3005,8 +3116,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -3022,8 +3134,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -3039,8 +3152,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -3056,8 +3170,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -3073,8 +3188,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -3090,8 +3206,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -3107,8 +3224,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -3124,8 +3242,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -3141,8 +3260,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -3158,8 +3278,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -3175,8 +3296,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -3192,8 +3314,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -3209,18 +3332,19 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
@@ -3253,7 +3377,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3263,9 +3387,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3278,6 +3402,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -3289,6 +3414,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -3300,6 +3426,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -3313,6 +3440,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -3333,6 +3461,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -3396,10 +3525,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -3417,8 +3551,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -3434,8 +3569,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -3451,8 +3587,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -3468,8 +3605,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -3485,8 +3623,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -3502,8 +3641,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -3519,8 +3659,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -3536,8 +3677,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -3553,8 +3695,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -3570,8 +3713,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -3587,8 +3731,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -3604,8 +3749,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -3621,8 +3767,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -3638,8 +3785,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -3655,8 +3803,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -3672,8 +3821,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -3689,8 +3839,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -3706,8 +3857,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -3723,8 +3875,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -3740,8 +3893,9 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="n">
@@ -3757,8 +3911,9 @@
       <c r="G30" s="31"/>
       <c r="H30" s="33"/>
       <c r="I30" s="33"/>
-      <c r="J30" s="30"/>
+      <c r="J30" s="33"/>
       <c r="K30" s="30"/>
+      <c r="L30" s="30"/>
     </row>
     <row r="31" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="n">
@@ -3774,8 +3929,9 @@
       <c r="G31" s="35"/>
       <c r="H31" s="37"/>
       <c r="I31" s="37"/>
-      <c r="J31" s="34"/>
+      <c r="J31" s="37"/>
       <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
     </row>
     <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="n">
@@ -3791,8 +3947,9 @@
       <c r="G32" s="31"/>
       <c r="H32" s="33"/>
       <c r="I32" s="33"/>
-      <c r="J32" s="30"/>
+      <c r="J32" s="33"/>
       <c r="K32" s="30"/>
+      <c r="L32" s="30"/>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="n">
@@ -3808,8 +3965,9 @@
       <c r="G33" s="35"/>
       <c r="H33" s="37"/>
       <c r="I33" s="37"/>
-      <c r="J33" s="34"/>
+      <c r="J33" s="37"/>
       <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
     </row>
     <row r="34" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="n">
@@ -3825,8 +3983,9 @@
       <c r="G34" s="31"/>
       <c r="H34" s="33"/>
       <c r="I34" s="33"/>
-      <c r="J34" s="30"/>
+      <c r="J34" s="33"/>
       <c r="K34" s="30"/>
+      <c r="L34" s="30"/>
     </row>
     <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="n">
@@ -3842,8 +4001,9 @@
       <c r="G35" s="35"/>
       <c r="H35" s="37"/>
       <c r="I35" s="37"/>
-      <c r="J35" s="34"/>
+      <c r="J35" s="37"/>
       <c r="K35" s="34"/>
+      <c r="L35" s="34"/>
     </row>
     <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="n">
@@ -3859,8 +4019,9 @@
       <c r="G36" s="31"/>
       <c r="H36" s="33"/>
       <c r="I36" s="33"/>
-      <c r="J36" s="30"/>
+      <c r="J36" s="33"/>
       <c r="K36" s="30"/>
+      <c r="L36" s="30"/>
     </row>
     <row r="37" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="n">
@@ -3876,18 +4037,19 @@
       <c r="G37" s="35"/>
       <c r="H37" s="37"/>
       <c r="I37" s="37"/>
-      <c r="J37" s="34"/>
+      <c r="J37" s="37"/>
       <c r="K37" s="34"/>
+      <c r="L37" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
@@ -4421,7 +4583,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -4431,9 +4593,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4446,6 +4608,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -4457,6 +4620,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -4468,6 +4632,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -4481,6 +4646,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -4501,6 +4667,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -4578,10 +4745,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -4597,8 +4769,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -4612,8 +4785,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -4627,8 +4801,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -4642,8 +4817,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -4657,8 +4833,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -4672,8 +4849,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -4687,8 +4865,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -4702,8 +4881,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -4717,8 +4897,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -4732,8 +4913,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -4747,8 +4929,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -4762,8 +4945,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -4777,8 +4961,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -4792,8 +4977,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -4807,8 +4993,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -4822,8 +5009,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -4837,8 +5025,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -4852,8 +5041,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -4867,8 +5057,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -4882,8 +5073,9 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="n">
@@ -4897,8 +5089,9 @@
       <c r="G30" s="31"/>
       <c r="H30" s="33"/>
       <c r="I30" s="33"/>
-      <c r="J30" s="30"/>
+      <c r="J30" s="33"/>
       <c r="K30" s="30"/>
+      <c r="L30" s="30"/>
     </row>
     <row r="31" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="n">
@@ -4912,8 +5105,9 @@
       <c r="G31" s="35"/>
       <c r="H31" s="37"/>
       <c r="I31" s="37"/>
-      <c r="J31" s="34"/>
+      <c r="J31" s="37"/>
       <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
     </row>
     <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="n">
@@ -4927,8 +5121,9 @@
       <c r="G32" s="31"/>
       <c r="H32" s="33"/>
       <c r="I32" s="33"/>
-      <c r="J32" s="30"/>
+      <c r="J32" s="33"/>
       <c r="K32" s="30"/>
+      <c r="L32" s="30"/>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="n">
@@ -4942,8 +5137,9 @@
       <c r="G33" s="35"/>
       <c r="H33" s="37"/>
       <c r="I33" s="37"/>
-      <c r="J33" s="34"/>
+      <c r="J33" s="37"/>
       <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
     </row>
     <row r="34" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="n">
@@ -4957,8 +5153,9 @@
       <c r="G34" s="31"/>
       <c r="H34" s="33"/>
       <c r="I34" s="33"/>
-      <c r="J34" s="30"/>
+      <c r="J34" s="33"/>
       <c r="K34" s="30"/>
+      <c r="L34" s="30"/>
     </row>
     <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="n">
@@ -4972,8 +5169,9 @@
       <c r="G35" s="35"/>
       <c r="H35" s="37"/>
       <c r="I35" s="37"/>
-      <c r="J35" s="34"/>
+      <c r="J35" s="37"/>
       <c r="K35" s="34"/>
+      <c r="L35" s="34"/>
     </row>
     <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="n">
@@ -4987,8 +5185,9 @@
       <c r="G36" s="31"/>
       <c r="H36" s="33"/>
       <c r="I36" s="33"/>
-      <c r="J36" s="30"/>
+      <c r="J36" s="33"/>
       <c r="K36" s="30"/>
+      <c r="L36" s="30"/>
     </row>
     <row r="37" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="n">
@@ -5002,8 +5201,9 @@
       <c r="G37" s="35"/>
       <c r="H37" s="37"/>
       <c r="I37" s="37"/>
-      <c r="J37" s="34"/>
+      <c r="J37" s="37"/>
       <c r="K37" s="34"/>
+      <c r="L37" s="34"/>
     </row>
     <row r="38" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="20" t="n">
@@ -5017,8 +5217,9 @@
       <c r="G38" s="31"/>
       <c r="H38" s="33"/>
       <c r="I38" s="33"/>
-      <c r="J38" s="30"/>
+      <c r="J38" s="33"/>
       <c r="K38" s="30"/>
+      <c r="L38" s="30"/>
     </row>
     <row r="39" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="n">
@@ -5032,18 +5233,19 @@
       <c r="G39" s="35"/>
       <c r="H39" s="37"/>
       <c r="I39" s="37"/>
-      <c r="J39" s="34"/>
+      <c r="J39" s="37"/>
       <c r="K39" s="34"/>
+      <c r="L39" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
@@ -5080,7 +5282,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -5090,9 +5292,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5105,6 +5307,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -5116,6 +5319,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -5127,6 +5331,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -5140,6 +5345,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -5160,6 +5366,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -5237,10 +5444,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -5256,8 +5468,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -5271,8 +5484,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -5286,8 +5500,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -5301,8 +5516,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -5316,8 +5532,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -5331,8 +5548,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -5346,8 +5564,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -5361,8 +5580,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -5376,8 +5596,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -5391,8 +5612,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -5406,8 +5628,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -5421,8 +5644,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -5436,8 +5660,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -5451,8 +5676,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -5466,8 +5692,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -5481,8 +5708,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -5496,8 +5724,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -5511,8 +5740,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -5526,8 +5756,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -5541,18 +5772,19 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
@@ -5589,7 +5821,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -5599,9 +5831,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5614,6 +5846,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -5625,6 +5858,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -5636,6 +5870,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -5649,6 +5884,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -5669,6 +5905,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -5746,10 +5983,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -5765,8 +6007,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -5780,8 +6023,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -5795,8 +6039,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -5810,8 +6055,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -5825,8 +6071,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -5840,8 +6087,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -5855,8 +6103,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -5870,8 +6119,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -5885,8 +6135,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -5900,8 +6151,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -5915,8 +6167,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -5930,8 +6183,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -5945,8 +6199,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -5960,8 +6215,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -5975,8 +6231,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -5990,8 +6247,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -6005,8 +6263,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -6020,8 +6279,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -6035,8 +6295,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -6050,8 +6311,9 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="n">
@@ -6065,8 +6327,9 @@
       <c r="G30" s="31"/>
       <c r="H30" s="33"/>
       <c r="I30" s="33"/>
-      <c r="J30" s="30"/>
+      <c r="J30" s="33"/>
       <c r="K30" s="30"/>
+      <c r="L30" s="30"/>
     </row>
     <row r="31" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="n">
@@ -6080,8 +6343,9 @@
       <c r="G31" s="35"/>
       <c r="H31" s="37"/>
       <c r="I31" s="37"/>
-      <c r="J31" s="34"/>
+      <c r="J31" s="37"/>
       <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
     </row>
     <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="n">
@@ -6095,8 +6359,9 @@
       <c r="G32" s="31"/>
       <c r="H32" s="33"/>
       <c r="I32" s="33"/>
-      <c r="J32" s="30"/>
+      <c r="J32" s="33"/>
       <c r="K32" s="30"/>
+      <c r="L32" s="30"/>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="n">
@@ -6110,8 +6375,9 @@
       <c r="G33" s="35"/>
       <c r="H33" s="37"/>
       <c r="I33" s="37"/>
-      <c r="J33" s="34"/>
+      <c r="J33" s="37"/>
       <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
     </row>
     <row r="34" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="n">
@@ -6125,8 +6391,9 @@
       <c r="G34" s="31"/>
       <c r="H34" s="33"/>
       <c r="I34" s="33"/>
-      <c r="J34" s="30"/>
+      <c r="J34" s="33"/>
       <c r="K34" s="30"/>
+      <c r="L34" s="30"/>
     </row>
     <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="n">
@@ -6140,8 +6407,9 @@
       <c r="G35" s="35"/>
       <c r="H35" s="37"/>
       <c r="I35" s="37"/>
-      <c r="J35" s="34"/>
+      <c r="J35" s="37"/>
       <c r="K35" s="34"/>
+      <c r="L35" s="34"/>
     </row>
     <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="n">
@@ -6155,8 +6423,9 @@
       <c r="G36" s="31"/>
       <c r="H36" s="33"/>
       <c r="I36" s="33"/>
-      <c r="J36" s="30"/>
+      <c r="J36" s="33"/>
       <c r="K36" s="30"/>
+      <c r="L36" s="30"/>
     </row>
     <row r="37" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="n">
@@ -6170,8 +6439,9 @@
       <c r="G37" s="35"/>
       <c r="H37" s="37"/>
       <c r="I37" s="37"/>
-      <c r="J37" s="34"/>
+      <c r="J37" s="37"/>
       <c r="K37" s="34"/>
+      <c r="L37" s="34"/>
     </row>
     <row r="38" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="20" t="n">
@@ -6185,8 +6455,9 @@
       <c r="G38" s="31"/>
       <c r="H38" s="33"/>
       <c r="I38" s="33"/>
-      <c r="J38" s="30"/>
+      <c r="J38" s="33"/>
       <c r="K38" s="30"/>
+      <c r="L38" s="30"/>
     </row>
     <row r="39" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="n">
@@ -6200,18 +6471,19 @@
       <c r="G39" s="35"/>
       <c r="H39" s="37"/>
       <c r="I39" s="37"/>
-      <c r="J39" s="34"/>
+      <c r="J39" s="37"/>
       <c r="K39" s="34"/>
+      <c r="L39" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
@@ -6248,7 +6520,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -6258,9 +6530,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6273,6 +6545,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -6284,6 +6557,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -6295,6 +6569,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -6308,6 +6583,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -6328,6 +6604,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -6405,10 +6682,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -6424,8 +6706,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -6439,8 +6722,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -6454,8 +6738,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -6469,8 +6754,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -6484,8 +6770,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -6499,8 +6786,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -6514,8 +6802,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -6529,8 +6818,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -6544,8 +6834,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -6559,8 +6850,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -6574,8 +6866,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -6589,8 +6882,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -6604,8 +6898,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -6619,8 +6914,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -6634,8 +6930,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -6649,8 +6946,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -6664,8 +6962,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -6679,8 +6978,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -6694,8 +6994,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -6709,8 +7010,9 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="n">
@@ -6724,8 +7026,9 @@
       <c r="G30" s="31"/>
       <c r="H30" s="33"/>
       <c r="I30" s="33"/>
-      <c r="J30" s="30"/>
+      <c r="J30" s="33"/>
       <c r="K30" s="30"/>
+      <c r="L30" s="30"/>
     </row>
     <row r="31" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="n">
@@ -6739,8 +7042,9 @@
       <c r="G31" s="35"/>
       <c r="H31" s="37"/>
       <c r="I31" s="37"/>
-      <c r="J31" s="34"/>
+      <c r="J31" s="37"/>
       <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
     </row>
     <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="n">
@@ -6754,8 +7058,9 @@
       <c r="G32" s="31"/>
       <c r="H32" s="33"/>
       <c r="I32" s="33"/>
-      <c r="J32" s="30"/>
+      <c r="J32" s="33"/>
       <c r="K32" s="30"/>
+      <c r="L32" s="30"/>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="n">
@@ -6769,8 +7074,9 @@
       <c r="G33" s="35"/>
       <c r="H33" s="37"/>
       <c r="I33" s="37"/>
-      <c r="J33" s="34"/>
+      <c r="J33" s="37"/>
       <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
     </row>
     <row r="34" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="n">
@@ -6784,8 +7090,9 @@
       <c r="G34" s="31"/>
       <c r="H34" s="33"/>
       <c r="I34" s="33"/>
-      <c r="J34" s="30"/>
+      <c r="J34" s="33"/>
       <c r="K34" s="30"/>
+      <c r="L34" s="30"/>
     </row>
     <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="n">
@@ -6799,8 +7106,9 @@
       <c r="G35" s="35"/>
       <c r="H35" s="37"/>
       <c r="I35" s="37"/>
-      <c r="J35" s="34"/>
+      <c r="J35" s="37"/>
       <c r="K35" s="34"/>
+      <c r="L35" s="34"/>
     </row>
     <row r="36" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="n">
@@ -6814,8 +7122,9 @@
       <c r="G36" s="31"/>
       <c r="H36" s="33"/>
       <c r="I36" s="33"/>
-      <c r="J36" s="30"/>
+      <c r="J36" s="33"/>
       <c r="K36" s="30"/>
+      <c r="L36" s="30"/>
     </row>
     <row r="37" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="n">
@@ -6829,8 +7138,9 @@
       <c r="G37" s="35"/>
       <c r="H37" s="37"/>
       <c r="I37" s="37"/>
-      <c r="J37" s="34"/>
+      <c r="J37" s="37"/>
       <c r="K37" s="34"/>
+      <c r="L37" s="34"/>
     </row>
     <row r="38" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="20" t="n">
@@ -6844,8 +7154,9 @@
       <c r="G38" s="31"/>
       <c r="H38" s="33"/>
       <c r="I38" s="33"/>
-      <c r="J38" s="30"/>
+      <c r="J38" s="33"/>
       <c r="K38" s="30"/>
+      <c r="L38" s="30"/>
     </row>
     <row r="39" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="n">
@@ -6859,18 +7170,19 @@
       <c r="G39" s="35"/>
       <c r="H39" s="37"/>
       <c r="I39" s="37"/>
-      <c r="J39" s="34"/>
+      <c r="J39" s="37"/>
       <c r="K39" s="34"/>
+      <c r="L39" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
@@ -6907,7 +7219,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -6917,9 +7229,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6932,6 +7244,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -6943,6 +7256,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -6954,6 +7268,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -6967,6 +7282,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -6987,6 +7303,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -7064,10 +7381,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -7083,8 +7405,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -7098,8 +7421,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -7113,8 +7437,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -7128,8 +7453,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -7143,8 +7469,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -7158,8 +7485,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -7173,8 +7501,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -7188,8 +7517,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -7203,8 +7533,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -7218,8 +7549,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -7233,8 +7565,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -7248,8 +7581,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -7263,8 +7597,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -7278,8 +7613,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -7293,8 +7629,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -7308,8 +7645,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -7323,8 +7661,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -7338,8 +7677,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -7353,8 +7693,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -7368,18 +7709,19 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
@@ -7416,7 +7758,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -7426,9 +7768,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7441,6 +7783,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -7452,6 +7795,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -7463,6 +7807,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -7476,6 +7821,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -7496,6 +7842,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -7573,10 +7920,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -7592,8 +7944,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -7607,8 +7960,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -7622,8 +7976,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -7637,8 +7992,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -7652,8 +8008,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -7667,8 +8024,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -7682,8 +8040,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -7697,8 +8056,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -7712,8 +8072,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -7727,8 +8088,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -7742,8 +8104,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -7757,8 +8120,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -7772,8 +8136,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -7787,8 +8152,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -7802,8 +8168,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -7817,8 +8184,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -7832,8 +8200,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -7847,8 +8216,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -7862,8 +8232,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -7877,18 +8248,19 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>
@@ -7925,7 +8297,7 @@
     <tabColor rgb="FF1B2A6B"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -7935,9 +8307,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7950,6 +8322,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C2" s="7" t="s">
@@ -7961,6 +8334,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="8" t="s">
@@ -7972,6 +8346,7 @@
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
@@ -7985,6 +8360,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
@@ -8005,6 +8381,7 @@
       <c r="I5" s="26"/>
       <c r="J5" s="27"/>
       <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
@@ -8068,10 +8445,15 @@
       <c r="I9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>جوال الطالب</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="L9" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -8089,8 +8471,9 @@
       <c r="G10" s="31"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
-      <c r="J10" s="30"/>
+      <c r="J10" s="33"/>
       <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
@@ -8106,8 +8489,9 @@
       <c r="G11" s="35"/>
       <c r="H11" s="37"/>
       <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
+      <c r="J11" s="37"/>
       <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
@@ -8123,8 +8507,9 @@
       <c r="G12" s="31"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
-      <c r="J12" s="30"/>
+      <c r="J12" s="33"/>
       <c r="K12" s="30"/>
+      <c r="L12" s="30"/>
     </row>
     <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
@@ -8140,8 +8525,9 @@
       <c r="G13" s="35"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
+      <c r="J13" s="37"/>
       <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
@@ -8157,8 +8543,9 @@
       <c r="G14" s="31"/>
       <c r="H14" s="33"/>
       <c r="I14" s="33"/>
-      <c r="J14" s="30"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
     </row>
     <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
@@ -8174,8 +8561,9 @@
       <c r="G15" s="35"/>
       <c r="H15" s="37"/>
       <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
+      <c r="J15" s="37"/>
       <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
     </row>
     <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="n">
@@ -8191,8 +8579,9 @@
       <c r="G16" s="31"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
-      <c r="J16" s="30"/>
+      <c r="J16" s="33"/>
       <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="n">
@@ -8208,8 +8597,9 @@
       <c r="G17" s="35"/>
       <c r="H17" s="37"/>
       <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
+      <c r="J17" s="37"/>
       <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="n">
@@ -8225,8 +8615,9 @@
       <c r="G18" s="31"/>
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
-      <c r="J18" s="30"/>
+      <c r="J18" s="33"/>
       <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="n">
@@ -8242,8 +8633,9 @@
       <c r="G19" s="35"/>
       <c r="H19" s="37"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
+      <c r="J19" s="37"/>
       <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -8259,8 +8651,9 @@
       <c r="G20" s="31"/>
       <c r="H20" s="33"/>
       <c r="I20" s="33"/>
-      <c r="J20" s="30"/>
+      <c r="J20" s="33"/>
       <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="n">
@@ -8276,8 +8669,9 @@
       <c r="G21" s="35"/>
       <c r="H21" s="37"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
+      <c r="J21" s="37"/>
       <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="n">
@@ -8293,8 +8687,9 @@
       <c r="G22" s="31"/>
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
-      <c r="J22" s="30"/>
+      <c r="J22" s="33"/>
       <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
     </row>
     <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="n">
@@ -8310,8 +8705,9 @@
       <c r="G23" s="35"/>
       <c r="H23" s="37"/>
       <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="n">
@@ -8327,8 +8723,9 @@
       <c r="G24" s="31"/>
       <c r="H24" s="33"/>
       <c r="I24" s="33"/>
-      <c r="J24" s="30"/>
+      <c r="J24" s="33"/>
       <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="n">
@@ -8344,8 +8741,9 @@
       <c r="G25" s="35"/>
       <c r="H25" s="37"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
+      <c r="J25" s="37"/>
       <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="n">
@@ -8361,8 +8759,9 @@
       <c r="G26" s="31"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="J26" s="30"/>
+      <c r="J26" s="33"/>
       <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="n">
@@ -8378,8 +8777,9 @@
       <c r="G27" s="35"/>
       <c r="H27" s="37"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
+      <c r="J27" s="37"/>
       <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="n">
@@ -8395,8 +8795,9 @@
       <c r="G28" s="31"/>
       <c r="H28" s="33"/>
       <c r="I28" s="33"/>
-      <c r="J28" s="30"/>
+      <c r="J28" s="33"/>
       <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
     </row>
     <row r="29" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="n">
@@ -8412,8 +8813,9 @@
       <c r="G29" s="35"/>
       <c r="H29" s="37"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
+      <c r="J29" s="37"/>
       <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
     </row>
     <row r="30" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="n">
@@ -8429,8 +8831,9 @@
       <c r="G30" s="31"/>
       <c r="H30" s="33"/>
       <c r="I30" s="33"/>
-      <c r="J30" s="30"/>
+      <c r="J30" s="33"/>
       <c r="K30" s="30"/>
+      <c r="L30" s="30"/>
     </row>
     <row r="31" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="n">
@@ -8446,8 +8849,9 @@
       <c r="G31" s="35"/>
       <c r="H31" s="37"/>
       <c r="I31" s="37"/>
-      <c r="J31" s="34"/>
+      <c r="J31" s="37"/>
       <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
     </row>
     <row r="32" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="n">
@@ -8463,8 +8867,9 @@
       <c r="G32" s="31"/>
       <c r="H32" s="33"/>
       <c r="I32" s="33"/>
-      <c r="J32" s="30"/>
+      <c r="J32" s="33"/>
       <c r="K32" s="30"/>
+      <c r="L32" s="30"/>
     </row>
     <row r="33" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="n">
@@ -8480,18 +8885,19 @@
       <c r="G33" s="35"/>
       <c r="H33" s="37"/>
       <c r="I33" s="37"/>
-      <c r="J33" s="34"/>
+      <c r="J33" s="37"/>
       <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="C3:I3"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A7:B7"/>

</xml_diff>